<commit_message>
fix: reconcile S04 hotel breakfast costing
</commit_message>
<xml_diff>
--- a/models/scenarios/S04/FINMODEL_VARSHAVKA_USALI_SCENARIO_S04_v3.0.0.xlsx
+++ b/models/scenarios/S04/FINMODEL_VARSHAVKA_USALI_SCENARIO_S04_v3.0.0.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_РЕЗЮМЕ" sheetId="1" r:id="Re2525fa93af049af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_ВВОД" sheetId="2" r:id="Re65e7300bb1a4ba8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_КАЛЕНДАРЬ" sheetId="3" r:id="R7d21da7248ca44a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ДОХОДЫ" sheetId="4" r:id="R8f18bb9aee194f78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_СЕБЕСТОИМОСТЬ" sheetId="5" r:id="R088b1277464646d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ФОТ" sheetId="6" r:id="Rbe29adf6e97f4e64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_OPEX_USALI" sheetId="7" r:id="R9a4e07866eb24581"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_PNL_НАЛОГИ" sheetId="8" r:id="R0fab9ec1c68841e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_ПРОВЕРКИ" sheetId="9" r:id="Rdacbef0476914dd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_СРАВНЕНИЕ_S03" sheetId="10" r:id="Rfae12e5c2a854ed2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_СРАВНЕНИЕ_S02_S03" sheetId="11" r:id="R71b2a0453a7948da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_ПОСУДА" sheetId="12" r:id="Rb2e347dcedb04c0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_ЦЕНТР_ИНВЕСТИЦИЙ" sheetId="13" r:id="Ra16fded4dc8242ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_ИЗМЕНЕНИЯ_v0.1.6" sheetId="14" r:id="R311d11fc60004cd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_ПРОГРАММА_КУХНИ" sheetId="15" r:id="R299d1ad4d64d4632"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_ЗАВТРАК_v0.1.7" sheetId="16" r:id="R3a35e0136e174d6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRICE_REGISTER" sheetId="17" r:id="Rbe6258e13d1f4778"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BREAKFAST_RECIPES" sheetId="18" r:id="R73d6ebf807894ee7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BREAKFAST_COSTING" sheetId="19" r:id="R4288819f90464d96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_РЕЗЮМЕ" sheetId="1" r:id="R3cc53e77eeaa4b28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_ВВОД" sheetId="2" r:id="R9675655050104c6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_КАЛЕНДАРЬ" sheetId="3" r:id="R6d9798d2f0c24602"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ДОХОДЫ" sheetId="4" r:id="Rb6271484db924eef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_СЕБЕСТОИМОСТЬ" sheetId="5" r:id="Rec4211d9005b4d70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ФОТ" sheetId="6" r:id="Rc49c72477519448b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_OPEX_USALI" sheetId="7" r:id="Rde5c5fc9b22346c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_PNL_НАЛОГИ" sheetId="8" r:id="Rc75166c094344089"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_ПРОВЕРКИ" sheetId="9" r:id="R39d25363f1e842c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_СРАВНЕНИЕ_S03" sheetId="10" r:id="Rd74500d19ef24be4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_СРАВНЕНИЕ_S02_S03" sheetId="11" r:id="R79c3c177083a4b66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_ПОСУДА" sheetId="12" r:id="Raafbaae6744048ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_ЦЕНТР_ИНВЕСТИЦИЙ" sheetId="13" r:id="Rc756436f718e433c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_ИЗМЕНЕНИЯ_v0.1.6" sheetId="14" r:id="R31e2448f5f634288"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_ПРОГРАММА_КУХНИ" sheetId="15" r:id="R360d384678de42f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_ЗАВТРАК_v0.1.7" sheetId="16" r:id="R429d4cb1f78f49a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRICE_REGISTER" sheetId="17" r:id="R7e4ca01d03914295"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BREAKFAST_RECIPES" sheetId="18" r:id="R9a206789cb3349cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BREAKFAST_COSTING" sheetId="19" r:id="Rc4b1744e419545f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1374,7 +1374,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1f5be9e6cc7b42e0"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra358c7c342f2476a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2765,7 +2765,7 @@
     <x:mergeCell ref="A36:F36"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b8e36ec07074b36"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42c38496af774cc9"/>
 </x:worksheet>
 </file>
 
@@ -5835,30 +5835,30 @@
     <x:mergeCell ref="B36:S36"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="Ra1763b22319a4949"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R437176a9101b4170"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="R35b579e2ad844a7c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="Rf3476e2aebbe4453"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="R4987840ba7184e84"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="R396ff0fe194c4c7c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="Ra826cf6bc5704988"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="R5482a07b47a64ce6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="R67ee80907a5042be"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="R1ac5dd510690474f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="R449c9c5354af4906"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="R688f42b97ba44af2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="R437fc9ee8647444f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="R5ead644d05294f8c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="R745636279c174a2b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="R867da3251bba43a0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="R1c95b559201a4067"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="R5e1c281a7fe64b54"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="Re10e0525fd6c4cec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="Rde0799e747b84264"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="R9cfc0dd9b13b4fc8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="R9b0e6050528846ef"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="R5e8a23e2047a47e0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="Ra275cf93482b4a8f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="R804ef11d6bb2409b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="Rd69421359c904cfd"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="R689d7d50b3fa4517"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="R384eb7299e034bc5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="R1cad656b13b7493c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="Rbf6d032a69074570"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="R608db1a948cd4c67"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="Rd51f5a75f11f47ed"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="R5cce8ac0a8c54e12"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="Rb472b08705e54992"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="R58e1fd4727d940e1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="R37227d9e151548a5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="Rbc4a04175b1142a5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="Ra0eb428614ed4201"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="R3782e991931f4559"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="R29d0bd18c93745ad"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="Rec2c686d646c49e1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="R222043a4a6d04e6f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="R5849c14ee47e4368"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="R8dd02fdbf5644723"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="R5aab34540fd846f6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="Rcb2eb3d2fe294e7d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="R8b16060e34a24592"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="R011e310bf1314089"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6140,9 +6140,9 @@
     <x:mergeCell ref="B15:H15"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="R7e35c91822474c08"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="R895c94f75182475c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="Rb6e0f45e6d464a08"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="Rea826dce32d94a80"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="Rd9b25599525b4772"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="Rfca40bdbfc4b42cc"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -10166,13 +10166,14 @@
         <x:v>Яйцо C0</x:v>
       </x:c>
       <x:c r="D4" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F4</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="E4" s="307" t="str">
         <x:v>шт.</x:v>
       </x:c>
       <x:c r="F4" s="307" t="n">
-        <x:f>PRICE_REGISTER!I4</x:f>
+        <x:f>'PRICE_REGISTER'!I4</x:f>
         <x:v>12.999</x:v>
       </x:c>
       <x:c r="G4" s="307" t="n">
@@ -10200,13 +10201,14 @@
         <x:v>Масло сливочное</x:v>
       </x:c>
       <x:c r="D5" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F5</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E5" s="307" t="str">
         <x:v>г</x:v>
       </x:c>
       <x:c r="F5" s="307" t="n">
-        <x:f>PRICE_REGISTER!I7</x:f>
+        <x:f>'PRICE_REGISTER'!I7</x:f>
         <x:v>1111.0555555555557</x:v>
       </x:c>
       <x:c r="G5" s="307" t="n">
@@ -10234,13 +10236,14 @@
         <x:v>Соль</x:v>
       </x:c>
       <x:c r="D6" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F6</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E6" s="307" t="str">
         <x:v>г</x:v>
       </x:c>
       <x:c r="F6" s="307" t="n">
-        <x:f>PRICE_REGISTER!I10</x:f>
+        <x:f>'PRICE_REGISTER'!I10</x:f>
         <x:v>42.99</x:v>
       </x:c>
       <x:c r="G6" s="307" t="n">
@@ -10268,13 +10271,14 @@
         <x:v>Меланж</x:v>
       </x:c>
       <x:c r="D7" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F7</x:f>
         <x:v>126</x:v>
       </x:c>
       <x:c r="E7" s="307" t="str">
         <x:v>г</x:v>
       </x:c>
       <x:c r="F7" s="307" t="n">
-        <x:f>PRICE_REGISTER!I5</x:f>
+        <x:f>'PRICE_REGISTER'!I5</x:f>
         <x:v>401.66666666666663</x:v>
       </x:c>
       <x:c r="G7" s="307" t="n">
@@ -10302,13 +10306,14 @@
         <x:v>Молоко</x:v>
       </x:c>
       <x:c r="D8" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F8</x:f>
         <x:v>50</x:v>
       </x:c>
       <x:c r="E8" s="307" t="str">
         <x:v>мл</x:v>
       </x:c>
       <x:c r="F8" s="307" t="n">
-        <x:f>PRICE_REGISTER!I6</x:f>
+        <x:f>'PRICE_REGISTER'!I6</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="G8" s="307" t="n">
@@ -10336,13 +10341,14 @@
         <x:v>Масло сливочное</x:v>
       </x:c>
       <x:c r="D9" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F9</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E9" s="307" t="str">
         <x:v>г</x:v>
       </x:c>
       <x:c r="F9" s="307" t="n">
-        <x:f>PRICE_REGISTER!I7</x:f>
+        <x:f>'PRICE_REGISTER'!I7</x:f>
         <x:v>1111.0555555555557</x:v>
       </x:c>
       <x:c r="G9" s="307" t="n">
@@ -10370,13 +10376,14 @@
         <x:v>Соль</x:v>
       </x:c>
       <x:c r="D10" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F10</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E10" s="307" t="str">
         <x:v>г</x:v>
       </x:c>
       <x:c r="F10" s="307" t="n">
-        <x:f>PRICE_REGISTER!I10</x:f>
+        <x:f>'PRICE_REGISTER'!I10</x:f>
         <x:v>42.99</x:v>
       </x:c>
       <x:c r="G10" s="307" t="n">
@@ -10404,13 +10411,14 @@
         <x:v>Овсяные хлопья</x:v>
       </x:c>
       <x:c r="D11" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F11</x:f>
         <x:v>45</x:v>
       </x:c>
       <x:c r="E11" s="307" t="str">
         <x:v>г</x:v>
       </x:c>
       <x:c r="F11" s="307" t="n">
-        <x:f>PRICE_REGISTER!I8</x:f>
+        <x:f>'PRICE_REGISTER'!I8</x:f>
         <x:v>209.98</x:v>
       </x:c>
       <x:c r="G11" s="307" t="n">
@@ -10438,13 +10446,14 @@
         <x:v>Молоко</x:v>
       </x:c>
       <x:c r="D12" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F12</x:f>
         <x:v>125</x:v>
       </x:c>
       <x:c r="E12" s="307" t="str">
         <x:v>мл</x:v>
       </x:c>
       <x:c r="F12" s="307" t="n">
-        <x:f>PRICE_REGISTER!I6</x:f>
+        <x:f>'PRICE_REGISTER'!I6</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="G12" s="307" t="n">
@@ -10472,6 +10481,7 @@
         <x:v>Вода</x:v>
       </x:c>
       <x:c r="D13" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F13</x:f>
         <x:v>100</x:v>
       </x:c>
       <x:c r="E13" s="307" t="str">
@@ -10505,13 +10515,14 @@
         <x:v>Сахар</x:v>
       </x:c>
       <x:c r="D14" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F14</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E14" s="307" t="str">
         <x:v>г</x:v>
       </x:c>
       <x:c r="F14" s="307" t="n">
-        <x:f>PRICE_REGISTER!I9</x:f>
+        <x:f>'PRICE_REGISTER'!I9</x:f>
         <x:v>99.99</x:v>
       </x:c>
       <x:c r="G14" s="307" t="n">
@@ -10539,13 +10550,14 @@
         <x:v>Масло сливочное</x:v>
       </x:c>
       <x:c r="D15" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F15</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E15" s="307" t="str">
         <x:v>г</x:v>
       </x:c>
       <x:c r="F15" s="307" t="n">
-        <x:f>PRICE_REGISTER!I7</x:f>
+        <x:f>'PRICE_REGISTER'!I7</x:f>
         <x:v>1111.0555555555557</x:v>
       </x:c>
       <x:c r="G15" s="307" t="n">
@@ -10573,13 +10585,14 @@
         <x:v>Соль</x:v>
       </x:c>
       <x:c r="D16" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F16</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E16" s="307" t="str">
         <x:v>г</x:v>
       </x:c>
       <x:c r="F16" s="307" t="n">
-        <x:f>PRICE_REGISTER!I10</x:f>
+        <x:f>'PRICE_REGISTER'!I10</x:f>
         <x:v>42.99</x:v>
       </x:c>
       <x:c r="G16" s="307" t="n">
@@ -10607,13 +10620,14 @@
         <x:v>Круассан 80 г</x:v>
       </x:c>
       <x:c r="D17" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F17</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E17" s="307" t="str">
         <x:v>шт.</x:v>
       </x:c>
       <x:c r="F17" s="307" t="n">
-        <x:f>PRICE_REGISTER!I11</x:f>
+        <x:f>'PRICE_REGISTER'!I11</x:f>
         <x:v>33.888</x:v>
       </x:c>
       <x:c r="G17" s="307" t="n">
@@ -10641,13 +10655,14 @@
         <x:v>Чеддер</x:v>
       </x:c>
       <x:c r="D18" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F18</x:f>
         <x:v>20</x:v>
       </x:c>
       <x:c r="E18" s="307" t="str">
         <x:v>г</x:v>
       </x:c>
       <x:c r="F18" s="307" t="n">
-        <x:f>PRICE_REGISTER!I12</x:f>
+        <x:f>'PRICE_REGISTER'!I12</x:f>
         <x:v>1399.92</x:v>
       </x:c>
       <x:c r="G18" s="307" t="n">
@@ -10675,13 +10690,14 @@
         <x:v>Fontina/Fontal</x:v>
       </x:c>
       <x:c r="D19" s="307" t="n">
+        <x:f>'BREAKFAST_RECIPES'!F19</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="E19" s="307" t="str">
         <x:v>г</x:v>
       </x:c>
       <x:c r="F19" s="307" t="n">
-        <x:f>PRICE_REGISTER!I13</x:f>
+        <x:f>'PRICE_REGISTER'!I13</x:f>
         <x:v>1800</x:v>
       </x:c>
       <x:c r="G19" s="307" t="n">
@@ -10774,7 +10790,7 @@
         <x:v>131.2826677777778</x:v>
       </x:c>
       <x:c r="F23" s="314" t="n">
-        <x:f>PRICE_REGISTER!I14</x:f>
+        <x:f>'PRICE_REGISTER'!I14</x:f>
         <x:v>60</x:v>
       </x:c>
       <x:c r="G23" s="314" t="n">
@@ -10812,7 +10828,7 @@
         <x:v>163.1946677777778</x:v>
       </x:c>
       <x:c r="F24" s="314" t="n">
-        <x:f>PRICE_REGISTER!I14</x:f>
+        <x:f>'PRICE_REGISTER'!I14</x:f>
         <x:v>60</x:v>
       </x:c>
       <x:c r="G24" s="314" t="n">
@@ -10850,7 +10866,7 @@
         <x:v>133.48371777777777</x:v>
       </x:c>
       <x:c r="F25" s="314" t="n">
-        <x:f>PRICE_REGISTER!I14</x:f>
+        <x:f>'PRICE_REGISTER'!I14</x:f>
         <x:v>60</x:v>
       </x:c>
       <x:c r="G25" s="314" t="n">
@@ -11008,13 +11024,13 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" style="174" customWidth="1"/>
-    <x:col min="2" max="2" width="19" style="174" customWidth="1"/>
-    <x:col min="3" max="3" width="42" style="174" customWidth="1"/>
+    <x:col min="1" max="1" width="34" style="174" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" style="174" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" style="174" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="16" style="174" customWidth="1"/>
     <x:col min="5" max="5" width="16" style="174" customWidth="1"/>
     <x:col min="6" max="6" width="18" style="174" customWidth="1"/>
-    <x:col min="7" max="7" width="48" style="174" customWidth="1"/>
+    <x:col min="7" max="7" width="54" style="174" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="174" customFormat="1" ht="28" customHeight="1">
@@ -15595,7 +15611,7 @@
         <x:v>Предварительно</x:v>
       </x:c>
       <x:c r="G147" s="270" t="str">
-        <x:v>Кухня 132,05 + напиток 60</x:v>
+        <x:v>Кухня 131,282668 + напиток 60</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
@@ -15619,7 +15635,7 @@
         <x:v>Предварительно</x:v>
       </x:c>
       <x:c r="G148" s="270" t="str">
-        <x:v>Кухня 138,50 + напиток 60</x:v>
+        <x:v>Кухня 163,194668 + напиток 60</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
@@ -15643,7 +15659,7 @@
         <x:v>Предварительно</x:v>
       </x:c>
       <x:c r="G149" s="270" t="str">
-        <x:v>Кухня 127,32 + напиток 60</x:v>
+        <x:v>Кухня 133,483718 + напиток 60</x:v>
       </x:c>
     </x:row>
     <x:row r="150">
@@ -58562,9 +58578,9 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" style="174" customWidth="1"/>
-    <x:col min="2" max="2" width="18" style="174" customWidth="1"/>
-    <x:col min="3" max="3" width="45" style="174" customWidth="1"/>
+    <x:col min="1" max="1" width="32" style="174" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" style="174" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="42" style="174" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="13" style="174" customWidth="1"/>
     <x:col min="5" max="5" width="13" style="174" customWidth="1"/>
     <x:col min="6" max="6" width="13" style="174" customWidth="1"/>
@@ -61676,6 +61692,630 @@
       </x:c>
       <x:c r="R46" t="str">
         <x:v>руб.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>МЕМО-КОНТУР ГОСТИНИЦА — ЗАВТРАКИ И УЖИНЫ УЧТЕНЫ В ИТОГАХ КАФЕ</x:v>
+      </x:c>
+      <x:c r="B48"/>
+      <x:c r="C48"/>
+      <x:c r="D48"/>
+      <x:c r="E48"/>
+      <x:c r="F48"/>
+      <x:c r="G48"/>
+      <x:c r="H48"/>
+      <x:c r="I48"/>
+      <x:c r="J48"/>
+      <x:c r="K48"/>
+      <x:c r="L48"/>
+      <x:c r="M48"/>
+      <x:c r="N48"/>
+      <x:c r="O48"/>
+      <x:c r="P48"/>
+      <x:c r="Q48"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>PNL.HOTEL.BREAKFAST.REV</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>Кафе — Гостиница</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>Выручка завтраков</x:v>
+      </x:c>
+      <x:c r="D49" t="n">
+        <x:f>'03_ДОХОДЫ'!D24</x:f>
+        <x:v>330000</x:v>
+      </x:c>
+      <x:c r="E49" t="n">
+        <x:f>'03_ДОХОДЫ'!E24</x:f>
+        <x:v>341000</x:v>
+      </x:c>
+      <x:c r="F49" t="n">
+        <x:f>'03_ДОХОДЫ'!F24</x:f>
+        <x:v>330000</x:v>
+      </x:c>
+      <x:c r="G49" t="n">
+        <x:f>'03_ДОХОДЫ'!G24</x:f>
+        <x:v>341000</x:v>
+      </x:c>
+      <x:c r="H49" t="n">
+        <x:f>'03_ДОХОДЫ'!H24</x:f>
+        <x:v>341000</x:v>
+      </x:c>
+      <x:c r="I49" t="n">
+        <x:f>'03_ДОХОДЫ'!I24</x:f>
+        <x:v>308000</x:v>
+      </x:c>
+      <x:c r="J49" t="n">
+        <x:f>'03_ДОХОДЫ'!J24</x:f>
+        <x:v>341000</x:v>
+      </x:c>
+      <x:c r="K49" t="n">
+        <x:f>'03_ДОХОДЫ'!K24</x:f>
+        <x:v>330000</x:v>
+      </x:c>
+      <x:c r="L49" t="n">
+        <x:f>'03_ДОХОДЫ'!L24</x:f>
+        <x:v>341000</x:v>
+      </x:c>
+      <x:c r="M49" t="n">
+        <x:f>'03_ДОХОДЫ'!M24</x:f>
+        <x:v>330000</x:v>
+      </x:c>
+      <x:c r="N49" t="n">
+        <x:f>'03_ДОХОДЫ'!N24</x:f>
+        <x:v>341000</x:v>
+      </x:c>
+      <x:c r="O49" t="n">
+        <x:f>'03_ДОХОДЫ'!O24</x:f>
+        <x:v>341000</x:v>
+      </x:c>
+      <x:c r="P49" t="n">
+        <x:f>SUM(D49:O49)</x:f>
+        <x:v>4015000</x:v>
+      </x:c>
+      <x:c r="Q49" t="n">
+        <x:f>AVERAGE(D49:O49)</x:f>
+        <x:v>334583.3333333333</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>PNL.HOTEL.BREAKFAST.COGS</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>Кафе — Гостиница</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>Прямой COGS завтраков</x:v>
+      </x:c>
+      <x:c r="D50" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!D15</x:f>
+        <x:v>122279.95816666666</x:v>
+      </x:c>
+      <x:c r="E50" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!E15</x:f>
+        <x:v>126355.95677222223</x:v>
+      </x:c>
+      <x:c r="F50" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!F15</x:f>
+        <x:v>122279.95816666666</x:v>
+      </x:c>
+      <x:c r="G50" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!G15</x:f>
+        <x:v>126355.95677222223</x:v>
+      </x:c>
+      <x:c r="H50" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!H15</x:f>
+        <x:v>126355.95677222223</x:v>
+      </x:c>
+      <x:c r="I50" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!I15</x:f>
+        <x:v>114127.96095555555</x:v>
+      </x:c>
+      <x:c r="J50" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!J15</x:f>
+        <x:v>126355.95677222223</x:v>
+      </x:c>
+      <x:c r="K50" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!K15</x:f>
+        <x:v>122279.95816666666</x:v>
+      </x:c>
+      <x:c r="L50" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!L15</x:f>
+        <x:v>126355.95677222223</x:v>
+      </x:c>
+      <x:c r="M50" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!M15</x:f>
+        <x:v>122279.95816666666</x:v>
+      </x:c>
+      <x:c r="N50" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!N15</x:f>
+        <x:v>126355.95677222223</x:v>
+      </x:c>
+      <x:c r="O50" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!O15</x:f>
+        <x:v>126355.95677222223</x:v>
+      </x:c>
+      <x:c r="P50" t="n">
+        <x:f>SUM(D50:O50)</x:f>
+        <x:v>1487739.4910277775</x:v>
+      </x:c>
+      <x:c r="Q50" t="n">
+        <x:f>AVERAGE(D50:O50)</x:f>
+        <x:v>123978.29091898147</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>PNL.HOTEL.BREAKFAST.CONTRIB</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>Кафе — Гостиница</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>Прямой результат завтраков</x:v>
+      </x:c>
+      <x:c r="D51" t="n">
+        <x:f>D49-D50</x:f>
+        <x:v>207720.04183333332</x:v>
+      </x:c>
+      <x:c r="E51" t="n">
+        <x:f>E49-E50</x:f>
+        <x:v>214644.04322777776</x:v>
+      </x:c>
+      <x:c r="F51" t="n">
+        <x:f>F49-F50</x:f>
+        <x:v>207720.04183333332</x:v>
+      </x:c>
+      <x:c r="G51" t="n">
+        <x:f>G49-G50</x:f>
+        <x:v>214644.04322777776</x:v>
+      </x:c>
+      <x:c r="H51" t="n">
+        <x:f>H49-H50</x:f>
+        <x:v>214644.04322777776</x:v>
+      </x:c>
+      <x:c r="I51" t="n">
+        <x:f>I49-I50</x:f>
+        <x:v>193872.03904444445</x:v>
+      </x:c>
+      <x:c r="J51" t="n">
+        <x:f>J49-J50</x:f>
+        <x:v>214644.04322777776</x:v>
+      </x:c>
+      <x:c r="K51" t="n">
+        <x:f>K49-K50</x:f>
+        <x:v>207720.04183333332</x:v>
+      </x:c>
+      <x:c r="L51" t="n">
+        <x:f>L49-L50</x:f>
+        <x:v>214644.04322777776</x:v>
+      </x:c>
+      <x:c r="M51" t="n">
+        <x:f>M49-M50</x:f>
+        <x:v>207720.04183333332</x:v>
+      </x:c>
+      <x:c r="N51" t="n">
+        <x:f>N49-N50</x:f>
+        <x:v>214644.04322777776</x:v>
+      </x:c>
+      <x:c r="O51" t="n">
+        <x:f>O49-O50</x:f>
+        <x:v>214644.04322777776</x:v>
+      </x:c>
+      <x:c r="P51" t="n">
+        <x:f>SUM(D51:O51)</x:f>
+        <x:v>2527260.5089722225</x:v>
+      </x:c>
+      <x:c r="Q51" t="n">
+        <x:f>AVERAGE(D51:O51)</x:f>
+        <x:v>210605.04241435186</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>PNL.HOTEL.DINNER.REV</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>Кафе — Гостиница</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>Выручка ужинов</x:v>
+      </x:c>
+      <x:c r="D52" t="n">
+        <x:f>'03_ДОХОДЫ'!D41</x:f>
+        <x:v>300000</x:v>
+      </x:c>
+      <x:c r="E52" t="n">
+        <x:f>'03_ДОХОДЫ'!E41</x:f>
+        <x:v>310000</x:v>
+      </x:c>
+      <x:c r="F52" t="n">
+        <x:f>'03_ДОХОДЫ'!F41</x:f>
+        <x:v>300000</x:v>
+      </x:c>
+      <x:c r="G52" t="n">
+        <x:f>'03_ДОХОДЫ'!G41</x:f>
+        <x:v>310000</x:v>
+      </x:c>
+      <x:c r="H52" t="n">
+        <x:f>'03_ДОХОДЫ'!H41</x:f>
+        <x:v>310000</x:v>
+      </x:c>
+      <x:c r="I52" t="n">
+        <x:f>'03_ДОХОДЫ'!I41</x:f>
+        <x:v>280000</x:v>
+      </x:c>
+      <x:c r="J52" t="n">
+        <x:f>'03_ДОХОДЫ'!J41</x:f>
+        <x:v>310000</x:v>
+      </x:c>
+      <x:c r="K52" t="n">
+        <x:f>'03_ДОХОДЫ'!K41</x:f>
+        <x:v>300000</x:v>
+      </x:c>
+      <x:c r="L52" t="n">
+        <x:f>'03_ДОХОДЫ'!L41</x:f>
+        <x:v>310000</x:v>
+      </x:c>
+      <x:c r="M52" t="n">
+        <x:f>'03_ДОХОДЫ'!M41</x:f>
+        <x:v>300000</x:v>
+      </x:c>
+      <x:c r="N52" t="n">
+        <x:f>'03_ДОХОДЫ'!N41</x:f>
+        <x:v>310000</x:v>
+      </x:c>
+      <x:c r="O52" t="n">
+        <x:f>'03_ДОХОДЫ'!O41</x:f>
+        <x:v>310000</x:v>
+      </x:c>
+      <x:c r="P52" t="n">
+        <x:f>SUM(D52:O52)</x:f>
+        <x:v>3650000</x:v>
+      </x:c>
+      <x:c r="Q52" t="n">
+        <x:f>AVERAGE(D52:O52)</x:f>
+        <x:v>304166.6666666667</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>PNL.HOTEL.DINNER.COGS</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>Кафе — Гостиница</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>Прямой COGS ужинов</x:v>
+      </x:c>
+      <x:c r="D53" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!D42</x:f>
+        <x:v>90000</x:v>
+      </x:c>
+      <x:c r="E53" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!E42</x:f>
+        <x:v>93000</x:v>
+      </x:c>
+      <x:c r="F53" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!F42</x:f>
+        <x:v>90000</x:v>
+      </x:c>
+      <x:c r="G53" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!G42</x:f>
+        <x:v>93000</x:v>
+      </x:c>
+      <x:c r="H53" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!H42</x:f>
+        <x:v>93000</x:v>
+      </x:c>
+      <x:c r="I53" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!I42</x:f>
+        <x:v>84000</x:v>
+      </x:c>
+      <x:c r="J53" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!J42</x:f>
+        <x:v>93000</x:v>
+      </x:c>
+      <x:c r="K53" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!K42</x:f>
+        <x:v>90000</x:v>
+      </x:c>
+      <x:c r="L53" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!L42</x:f>
+        <x:v>93000</x:v>
+      </x:c>
+      <x:c r="M53" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!M42</x:f>
+        <x:v>90000</x:v>
+      </x:c>
+      <x:c r="N53" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!N42</x:f>
+        <x:v>93000</x:v>
+      </x:c>
+      <x:c r="O53" t="n">
+        <x:f>'04_СЕБЕСТОИМОСТЬ'!O42</x:f>
+        <x:v>93000</x:v>
+      </x:c>
+      <x:c r="P53" t="n">
+        <x:f>SUM(D53:O53)</x:f>
+        <x:v>1095000</x:v>
+      </x:c>
+      <x:c r="Q53" t="n">
+        <x:f>AVERAGE(D53:O53)</x:f>
+        <x:v>91250</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>PNL.HOTEL.DINNER.CONTRIB</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>Кафе — Гостиница</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>Прямой результат ужинов</x:v>
+      </x:c>
+      <x:c r="D54" t="n">
+        <x:f>D52-D53</x:f>
+        <x:v>210000</x:v>
+      </x:c>
+      <x:c r="E54" t="n">
+        <x:f>E52-E53</x:f>
+        <x:v>217000</x:v>
+      </x:c>
+      <x:c r="F54" t="n">
+        <x:f>F52-F53</x:f>
+        <x:v>210000</x:v>
+      </x:c>
+      <x:c r="G54" t="n">
+        <x:f>G52-G53</x:f>
+        <x:v>217000</x:v>
+      </x:c>
+      <x:c r="H54" t="n">
+        <x:f>H52-H53</x:f>
+        <x:v>217000</x:v>
+      </x:c>
+      <x:c r="I54" t="n">
+        <x:f>I52-I53</x:f>
+        <x:v>196000</x:v>
+      </x:c>
+      <x:c r="J54" t="n">
+        <x:f>J52-J53</x:f>
+        <x:v>217000</x:v>
+      </x:c>
+      <x:c r="K54" t="n">
+        <x:f>K52-K53</x:f>
+        <x:v>210000</x:v>
+      </x:c>
+      <x:c r="L54" t="n">
+        <x:f>L52-L53</x:f>
+        <x:v>217000</x:v>
+      </x:c>
+      <x:c r="M54" t="n">
+        <x:f>M52-M53</x:f>
+        <x:v>210000</x:v>
+      </x:c>
+      <x:c r="N54" t="n">
+        <x:f>N52-N53</x:f>
+        <x:v>217000</x:v>
+      </x:c>
+      <x:c r="O54" t="n">
+        <x:f>O52-O53</x:f>
+        <x:v>217000</x:v>
+      </x:c>
+      <x:c r="P54" t="n">
+        <x:f>SUM(D54:O54)</x:f>
+        <x:v>2555000</x:v>
+      </x:c>
+      <x:c r="Q54" t="n">
+        <x:f>AVERAGE(D54:O54)</x:f>
+        <x:v>212916.66666666666</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>PNL.HOTEL.TOTAL.REV</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>Кафе — Гостиница</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>Итого выручка направления</x:v>
+      </x:c>
+      <x:c r="D55" t="n">
+        <x:f>D49+D52</x:f>
+        <x:v>630000</x:v>
+      </x:c>
+      <x:c r="E55" t="n">
+        <x:f>E49+E52</x:f>
+        <x:v>651000</x:v>
+      </x:c>
+      <x:c r="F55" t="n">
+        <x:f>F49+F52</x:f>
+        <x:v>630000</x:v>
+      </x:c>
+      <x:c r="G55" t="n">
+        <x:f>G49+G52</x:f>
+        <x:v>651000</x:v>
+      </x:c>
+      <x:c r="H55" t="n">
+        <x:f>H49+H52</x:f>
+        <x:v>651000</x:v>
+      </x:c>
+      <x:c r="I55" t="n">
+        <x:f>I49+I52</x:f>
+        <x:v>588000</x:v>
+      </x:c>
+      <x:c r="J55" t="n">
+        <x:f>J49+J52</x:f>
+        <x:v>651000</x:v>
+      </x:c>
+      <x:c r="K55" t="n">
+        <x:f>K49+K52</x:f>
+        <x:v>630000</x:v>
+      </x:c>
+      <x:c r="L55" t="n">
+        <x:f>L49+L52</x:f>
+        <x:v>651000</x:v>
+      </x:c>
+      <x:c r="M55" t="n">
+        <x:f>M49+M52</x:f>
+        <x:v>630000</x:v>
+      </x:c>
+      <x:c r="N55" t="n">
+        <x:f>N49+N52</x:f>
+        <x:v>651000</x:v>
+      </x:c>
+      <x:c r="O55" t="n">
+        <x:f>O49+O52</x:f>
+        <x:v>651000</x:v>
+      </x:c>
+      <x:c r="P55" t="n">
+        <x:f>SUM(D55:O55)</x:f>
+        <x:v>7665000</x:v>
+      </x:c>
+      <x:c r="Q55" t="n">
+        <x:f>AVERAGE(D55:O55)</x:f>
+        <x:v>638750</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
+        <x:v>PNL.HOTEL.TOTAL.COGS</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>Кафе — Гостиница</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>Итого прямой COGS направления</x:v>
+      </x:c>
+      <x:c r="D56" t="n">
+        <x:f>D50+D53</x:f>
+        <x:v>212279.95816666668</x:v>
+      </x:c>
+      <x:c r="E56" t="n">
+        <x:f>E50+E53</x:f>
+        <x:v>219355.95677222224</x:v>
+      </x:c>
+      <x:c r="F56" t="n">
+        <x:f>F50+F53</x:f>
+        <x:v>212279.95816666668</x:v>
+      </x:c>
+      <x:c r="G56" t="n">
+        <x:f>G50+G53</x:f>
+        <x:v>219355.95677222224</x:v>
+      </x:c>
+      <x:c r="H56" t="n">
+        <x:f>H50+H53</x:f>
+        <x:v>219355.95677222224</x:v>
+      </x:c>
+      <x:c r="I56" t="n">
+        <x:f>I50+I53</x:f>
+        <x:v>198127.96095555555</x:v>
+      </x:c>
+      <x:c r="J56" t="n">
+        <x:f>J50+J53</x:f>
+        <x:v>219355.95677222224</x:v>
+      </x:c>
+      <x:c r="K56" t="n">
+        <x:f>K50+K53</x:f>
+        <x:v>212279.95816666668</x:v>
+      </x:c>
+      <x:c r="L56" t="n">
+        <x:f>L50+L53</x:f>
+        <x:v>219355.95677222224</x:v>
+      </x:c>
+      <x:c r="M56" t="n">
+        <x:f>M50+M53</x:f>
+        <x:v>212279.95816666668</x:v>
+      </x:c>
+      <x:c r="N56" t="n">
+        <x:f>N50+N53</x:f>
+        <x:v>219355.95677222224</x:v>
+      </x:c>
+      <x:c r="O56" t="n">
+        <x:f>O50+O53</x:f>
+        <x:v>219355.95677222224</x:v>
+      </x:c>
+      <x:c r="P56" t="n">
+        <x:f>SUM(D56:O56)</x:f>
+        <x:v>2582739.4910277775</x:v>
+      </x:c>
+      <x:c r="Q56" t="n">
+        <x:f>AVERAGE(D56:O56)</x:f>
+        <x:v>215228.29091898145</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="str">
+        <x:v>PNL.HOTEL.TOTAL.CONTRIB</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>Кафе — Гостиница</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>Итого прямой результат направления</x:v>
+      </x:c>
+      <x:c r="D57" t="n">
+        <x:f>D55-D56</x:f>
+        <x:v>417720.0418333333</x:v>
+      </x:c>
+      <x:c r="E57" t="n">
+        <x:f>E55-E56</x:f>
+        <x:v>431644.04322777776</x:v>
+      </x:c>
+      <x:c r="F57" t="n">
+        <x:f>F55-F56</x:f>
+        <x:v>417720.0418333333</x:v>
+      </x:c>
+      <x:c r="G57" t="n">
+        <x:f>G55-G56</x:f>
+        <x:v>431644.04322777776</x:v>
+      </x:c>
+      <x:c r="H57" t="n">
+        <x:f>H55-H56</x:f>
+        <x:v>431644.04322777776</x:v>
+      </x:c>
+      <x:c r="I57" t="n">
+        <x:f>I55-I56</x:f>
+        <x:v>389872.03904444445</x:v>
+      </x:c>
+      <x:c r="J57" t="n">
+        <x:f>J55-J56</x:f>
+        <x:v>431644.04322777776</x:v>
+      </x:c>
+      <x:c r="K57" t="n">
+        <x:f>K55-K56</x:f>
+        <x:v>417720.0418333333</x:v>
+      </x:c>
+      <x:c r="L57" t="n">
+        <x:f>L55-L56</x:f>
+        <x:v>431644.04322777776</x:v>
+      </x:c>
+      <x:c r="M57" t="n">
+        <x:f>M55-M56</x:f>
+        <x:v>417720.0418333333</x:v>
+      </x:c>
+      <x:c r="N57" t="n">
+        <x:f>N55-N56</x:f>
+        <x:v>431644.04322777776</x:v>
+      </x:c>
+      <x:c r="O57" t="n">
+        <x:f>O55-O56</x:f>
+        <x:v>431644.04322777776</x:v>
+      </x:c>
+      <x:c r="P57" t="n">
+        <x:f>SUM(D57:O57)</x:f>
+        <x:v>5082260.508972222</x:v>
+      </x:c>
+      <x:c r="Q57" t="n">
+        <x:f>AVERAGE(D57:O57)</x:f>
+        <x:v>423521.7090810185</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -61709,13 +62349,13 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" style="174" customWidth="1"/>
-    <x:col min="2" max="2" width="42" style="174" customWidth="1"/>
+    <x:col min="1" max="1" width="32" style="174" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="46" style="174" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="16" style="174" customWidth="1"/>
     <x:col min="4" max="4" width="16" style="174" customWidth="1"/>
     <x:col min="5" max="5" width="16" style="174" customWidth="1"/>
     <x:col min="6" max="6" width="14" style="174" customWidth="1"/>
-    <x:col min="7" max="7" width="42" style="174" customWidth="1"/>
+    <x:col min="7" max="7" width="72" style="174" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="174" customFormat="1" ht="28" customHeight="1">
@@ -62918,19 +63558,45 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="D46" t="n">
-        <x:f>ABS('01_ВВОД'!$D$156-22)+ABS('01_ВВОД'!$D$157-21)</x:f>
-        <x:v>0</x:v>
+        <x:f>ABS('01_ВВОД'!$D$156-22)+ABS('01_ВВОД'!$D$157-21)+ABS('01_ВВОД'!$D$158-20)+ABS('03_ДОХОДЫ'!$P$22-7300)+ABS('04_СЕБЕСТОИМОСТЬ'!$P$15-'03_ДОХОДЫ'!$P$22*'01_ВВОД'!$D$142)</x:f>
+        <x:v>2.3283064365386963e-10</x:v>
       </x:c>
       <x:c r="E46" t="n">
         <x:f>D46-C46</x:f>
-        <x:v>0</x:v>
+        <x:v>2.3283064365386963e-10</x:v>
       </x:c>
       <x:c r="F46" t="str">
         <x:f>IF(ABS(E46)&lt;0.0001,"OK","ОШИБКА")</x:f>
         <x:v>OK</x:v>
       </x:c>
       <x:c r="G46" t="str">
-        <x:v>22 и 21 комплекс без повторного резерва</x:v>
+        <x:v>20 оплачиваемых обслуживаний; выпуск 22/21; финансовый COGS только для 7 300 оплаченных завтраков</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>CHK.BREAKFAST.NORMS</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>Нормы калькуляции равны BREAKFAST_RECIPES</x:v>
+      </x:c>
+      <x:c r="C47" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D47" t="n">
+        <x:f>ABS('BREAKFAST_COSTING'!D4-'BREAKFAST_RECIPES'!F4)+ABS('BREAKFAST_COSTING'!D5-'BREAKFAST_RECIPES'!F5)+ABS('BREAKFAST_COSTING'!D6-'BREAKFAST_RECIPES'!F6)+ABS('BREAKFAST_COSTING'!D7-'BREAKFAST_RECIPES'!F7)+ABS('BREAKFAST_COSTING'!D8-'BREAKFAST_RECIPES'!F8)+ABS('BREAKFAST_COSTING'!D9-'BREAKFAST_RECIPES'!F9)+ABS('BREAKFAST_COSTING'!D10-'BREAKFAST_RECIPES'!F10)+ABS('BREAKFAST_COSTING'!D11-'BREAKFAST_RECIPES'!F11)+ABS('BREAKFAST_COSTING'!D12-'BREAKFAST_RECIPES'!F12)+ABS('BREAKFAST_COSTING'!D13-'BREAKFAST_RECIPES'!F13)+ABS('BREAKFAST_COSTING'!D14-'BREAKFAST_RECIPES'!F14)+ABS('BREAKFAST_COSTING'!D15-'BREAKFAST_RECIPES'!F15)+ABS('BREAKFAST_COSTING'!D16-'BREAKFAST_RECIPES'!F16)+ABS('BREAKFAST_COSTING'!D17-'BREAKFAST_RECIPES'!F17)+ABS('BREAKFAST_COSTING'!D18-'BREAKFAST_RECIPES'!F18)+ABS('BREAKFAST_COSTING'!D19-'BREAKFAST_RECIPES'!F19)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E47" t="n">
+        <x:f>D47-C47</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F47" t="str">
+        <x:f>IF(ABS(E47)&lt;0.0001,"OK","ОШИБКА")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G47" t="str">
+        <x:v>D4:D19 связаны формулами с BREAKFAST_RECIPES!F4:F19</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Document Issue 52 control criteria
</commit_message>
<xml_diff>
--- a/models/scenarios/S04/FINMODEL_VARSHAVKA_USALI_SCENARIO_S04_v3.0.0.xlsx
+++ b/models/scenarios/S04/FINMODEL_VARSHAVKA_USALI_SCENARIO_S04_v3.0.0.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_РЕЗЮМЕ" sheetId="1" r:id="R3cc53e77eeaa4b28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_ВВОД" sheetId="2" r:id="R9675655050104c6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_КАЛЕНДАРЬ" sheetId="3" r:id="R6d9798d2f0c24602"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ДОХОДЫ" sheetId="4" r:id="Rb6271484db924eef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_СЕБЕСТОИМОСТЬ" sheetId="5" r:id="Rec4211d9005b4d70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ФОТ" sheetId="6" r:id="Rc49c72477519448b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_OPEX_USALI" sheetId="7" r:id="Rde5c5fc9b22346c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_PNL_НАЛОГИ" sheetId="8" r:id="Rc75166c094344089"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_ПРОВЕРКИ" sheetId="9" r:id="R39d25363f1e842c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_СРАВНЕНИЕ_S03" sheetId="10" r:id="Rd74500d19ef24be4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_СРАВНЕНИЕ_S02_S03" sheetId="11" r:id="R79c3c177083a4b66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_ПОСУДА" sheetId="12" r:id="Raafbaae6744048ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_ЦЕНТР_ИНВЕСТИЦИЙ" sheetId="13" r:id="Rc756436f718e433c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_ИЗМЕНЕНИЯ_v0.1.6" sheetId="14" r:id="R31e2448f5f634288"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_ПРОГРАММА_КУХНИ" sheetId="15" r:id="R360d384678de42f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_ЗАВТРАК_v0.1.7" sheetId="16" r:id="R429d4cb1f78f49a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRICE_REGISTER" sheetId="17" r:id="R7e4ca01d03914295"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BREAKFAST_RECIPES" sheetId="18" r:id="R9a206789cb3349cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BREAKFAST_COSTING" sheetId="19" r:id="Rc4b1744e419545f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_РЕЗЮМЕ" sheetId="1" r:id="Rc4f31b82db464ae2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_ВВОД" sheetId="2" r:id="R76a40a4cfa80478e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_КАЛЕНДАРЬ" sheetId="3" r:id="R8652293d112149c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_ДОХОДЫ" sheetId="4" r:id="R4b9f504998bc4c4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_СЕБЕСТОИМОСТЬ" sheetId="5" r:id="Rb6d0239267de49b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ФОТ" sheetId="6" r:id="R47257e3cdade42bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_OPEX_USALI" sheetId="7" r:id="Rfe9c3c27b36647e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_PNL_НАЛОГИ" sheetId="8" r:id="R7d7ed9365fbf43ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_ПРОВЕРКИ" sheetId="9" r:id="R57b9c322c6cb4431"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_СРАВНЕНИЕ_S03" sheetId="10" r:id="R3fb6e06265b14d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_СРАВНЕНИЕ_S02_S03" sheetId="11" r:id="Rbb0af998cc37428d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_ПОСУДА" sheetId="12" r:id="Rf35db32f02034f21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_ЦЕНТР_ИНВЕСТИЦИЙ" sheetId="13" r:id="Rd86ae3fb167440f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_ИЗМЕНЕНИЯ_v0.1.6" sheetId="14" r:id="R80be93f41cdb4a4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_ПРОГРАММА_КУХНИ" sheetId="15" r:id="R42e3406de9894a40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_ЗАВТРАК_v0.1.7" sheetId="16" r:id="Rd4cfe7963bcb4e28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRICE_REGISTER" sheetId="17" r:id="R93d4a0d3199a42b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BREAKFAST_RECIPES" sheetId="18" r:id="Rbaabd0df7503479a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BREAKFAST_COSTING" sheetId="19" r:id="Rd043662a5de647fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -365,7 +365,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="315">
+  <x:cellXfs count="316">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
@@ -1023,6 +1023,9 @@
     <x:xf numFmtId="211" fontId="24" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1374,7 +1377,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra358c7c342f2476a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R43f1ce5e7f894488"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2765,7 +2768,7 @@
     <x:mergeCell ref="A36:F36"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42c38496af774cc9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re71dfff2aed147d0"/>
 </x:worksheet>
 </file>
 
@@ -5835,30 +5838,30 @@
     <x:mergeCell ref="B36:S36"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="R804ef11d6bb2409b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="Rd69421359c904cfd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="R689d7d50b3fa4517"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="R384eb7299e034bc5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="R1cad656b13b7493c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="Rbf6d032a69074570"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="R608db1a948cd4c67"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="Rd51f5a75f11f47ed"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="R5cce8ac0a8c54e12"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="Rb472b08705e54992"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="R58e1fd4727d940e1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="R37227d9e151548a5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="Rbc4a04175b1142a5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="Ra0eb428614ed4201"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="R3782e991931f4559"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="R29d0bd18c93745ad"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="Rec2c686d646c49e1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="R222043a4a6d04e6f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="R5849c14ee47e4368"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="R8dd02fdbf5644723"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="R5aab34540fd846f6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="Rcb2eb3d2fe294e7d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="R8b16060e34a24592"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="R011e310bf1314089"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="R01bbe2f09f914c6a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="R7002601bd52d479b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="R604414e8e255487a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="Rb64a22ba21c44df8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="Rb441f6dbca694d39"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="R4caffbc1621148d3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="R722c942c169343c8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="Rb553efc92fca4f77"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="Rdf91907ede244fed"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="R85f3fb8d397947f6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="Ra332e7d73cbe409a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="R2aa9027851044aa1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="Ra3a1616bd9a34cf0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="Rf11a858aef844803"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="R647feed897474013"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="Rd20d7acc4d1c4167"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="R8b671d4d3cab4e4b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="R763ec2b863b0488e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="Rd08e16e847b54994"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S25" r:id="Rf64888177d454772"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="R5eeb477197a94c7b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="R5e04322594944fd8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="R5fe842cc76784964"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="R261d6a90b7364fb8"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6140,9 +6143,9 @@
     <x:mergeCell ref="B15:H15"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="Rea826dce32d94a80"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="Rd9b25599525b4772"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="Rfca40bdbfc4b42cc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="R38b348f50d364084"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="Rb799e9143b0e45fb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="R11b10052c1684b46"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -9816,10 +9819,10 @@
         <x:v>каша</x:v>
       </x:c>
       <x:c r="J12" s="309" t="n">
-        <x:v>111</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="K12" s="272" t="str">
-        <x:v>Стоимость по литрам; масса нетто требует КП</x:v>
+        <x:v>Аналитическое распределение выхода; стоимость по брутто 125 мл</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -9851,10 +9854,10 @@
         <x:v>каша</x:v>
       </x:c>
       <x:c r="J13" s="309" t="n">
-        <x:v>88</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="K13" s="272" t="str">
-        <x:v>Коммунальный ресурс; продуктовая стоимость 0</x:v>
+        <x:v>Аналитическое распределение выхода; коммунальный ресурс, стоимость 0</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -9886,9 +9889,11 @@
         <x:v>каша</x:v>
       </x:c>
       <x:c r="J14" s="309" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="K14" s="272" t="str"/>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K14" s="272" t="str">
+        <x:v>Аналитическое распределение готового выхода</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="272" t="str">
@@ -9919,9 +9924,11 @@
         <x:v>каша</x:v>
       </x:c>
       <x:c r="J15" s="309" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="K15" s="272" t="str"/>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K15" s="272" t="str">
+        <x:v>Аналитическое распределение готового выхода</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="272" t="str">
@@ -63599,6 +63606,32 @@
         <x:v>D4:D19 связаны формулами с BREAKFAST_RECIPES!F4:F19</x:v>
       </x:c>
     </x:row>
+    <x:row r="48" ht="44" customHeight="1">
+      <x:c r="A48" s="315" t="str">
+        <x:v>CHK.BREAKFAST.OATMEAL_250</x:v>
+      </x:c>
+      <x:c r="B48" s="315" t="str">
+        <x:v>Сумма аналитических выходов овсяной каши равна 250 г</x:v>
+      </x:c>
+      <x:c r="C48" s="315" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D48" s="315" t="n">
+        <x:f>ABS(SUM('BREAKFAST_RECIPES'!J11:J16)-250)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E48" s="315" t="n">
+        <x:f>D48-C48</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F48" s="315" t="str">
+        <x:f>IF(ABS(E48)&lt;0.0001,"OK","ОШИБКА")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="G48" s="315" t="str">
+        <x:v>BREAKFAST_RECIPES!J11:J16 = 45 + 108 + 86 + 5 + 5 + 1 = 250 г; брутто F11:F16 не изменяется</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A20:G20"/>

</xml_diff>